<commit_message>
Add Appium mobile automation framework, 440 E2E test cases, and GitHub Pages report pipeline
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Failed Test Cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Failed Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41,8 +41,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
   </fills>
@@ -456,12 +456,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Status</t>
         </is>
       </c>
     </row>

</xml_diff>